<commit_message>
Actualizar documentación presentación hito 2 - semana 10
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/Ev. Product Backlog.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/Ev. Product Backlog.xlsx
@@ -15,11 +15,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={bd851e13-179a-4533-bcc3-ad19a178ccfc}</author>
-    <author>tc={c26be8d4-2204-42ee-91d1-6496fb84b226}</author>
+    <author>tc={22a33020-94ca-405d-b52d-f5563f0938a4}</author>
+    <author>tc={32d35ea2-5a02-472b-9436-72eda681c8bd}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{bd851e13-179a-4533-bcc3-ad19a178ccfc}" ref="E1">
+    <comment authorId="0" xr:uid="{22a33020-94ca-405d-b52d-f5563f0938a4}" ref="E1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -28,7 +28,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{c26be8d4-2204-42ee-91d1-6496fb84b226}" ref="B1">
+    <comment authorId="1" xr:uid="{32d35ea2-5a02-472b-9436-72eda681c8bd}" ref="B1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -314,16 +314,16 @@
     <t>Campo de notas detalladas por tarea</t>
   </si>
   <si>
+    <t>Desarrollo de registro y asignación de labores por trabajador</t>
+  </si>
+  <si>
+    <t>H-10</t>
+  </si>
+  <si>
+    <t>Módulo de asignación de mano de obra</t>
+  </si>
+  <si>
     <t>En Progreso</t>
-  </si>
-  <si>
-    <t>Desarrollo de registro y asignación de labores por trabajador</t>
-  </si>
-  <si>
-    <t>H-10</t>
-  </si>
-  <si>
-    <t>Módulo de asignación de mano de obra</t>
   </si>
   <si>
     <t>Asignación de tareas por trabajador (visualización de los pedidos asignados)</t>
@@ -515,7 +515,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="SMOLENKS JOHAN ARAVENA CARVAJAL" id="{acbfa28a-a64c-49bb-a900-99c51bcfdfc1}" providerId="google-sheets"/>
+  <x18tc:person displayName="SMOLENKS JOHAN ARAVENA CARVAJAL" id="{fbfe4390-fc9b-46e4-aabe-2d249994f862}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -715,10 +715,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="B1" dT="2026-09-13T21:27:38.00" personId="{acbfa28a-a64c-49bb-a900-99c51bcfdfc1}" id="{c26be8d4-2204-42ee-91d1-6496fb84b226}" done="1">
+  <x18tc:threadedComment ref="B1" dT="2026-09-13T21:27:38.00" personId="{fbfe4390-fc9b-46e4-aabe-2d249994f862}" id="{32d35ea2-5a02-472b-9436-72eda681c8bd}" done="1">
     <x18tc:text xml:space="preserve">eliminar los que no aplican y cambiar redaccion</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="E1" dT="2026-09-13T21:27:43.00" personId="{acbfa28a-a64c-49bb-a900-99c51bcfdfc1}" id="{bd851e13-179a-4533-bcc3-ad19a178ccfc}" done="1">
+  <x18tc:threadedComment ref="E1" dT="2026-09-13T21:27:43.00" personId="{fbfe4390-fc9b-46e4-aabe-2d249994f862}" id="{22a33020-94ca-405d-b52d-f5563f0938a4}" done="1">
     <x18tc:text xml:space="preserve">eliminar los que no aplican y cambiar redaccion</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -1627,7 +1627,7 @@
         <v>20</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>90</v>
+        <v>13</v>
       </c>
       <c r="H32" s="3">
         <f t="shared" si="2"/>
@@ -1640,22 +1640,22 @@
         <v>P-32</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>73</v>
       </c>
       <c r="D33" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="F33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>90</v>
       </c>
       <c r="H33" s="3">
         <f t="shared" si="2"/>
@@ -1711,7 +1711,7 @@
         <v>12</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H35" s="3">
         <f t="shared" si="2"/>
@@ -1739,7 +1739,7 @@
         <v>12</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H36" s="3">
         <f t="shared" si="2"/>

</xml_diff>

<commit_message>
Actualizar documentación del Sprint 2 y corregir ortografía y redacción
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/Ev. Product Backlog.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/Ev. Product Backlog.xlsx
@@ -15,11 +15,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={22a33020-94ca-405d-b52d-f5563f0938a4}</author>
-    <author>tc={32d35ea2-5a02-472b-9436-72eda681c8bd}</author>
+    <author>tc={04b0f02b-9ddd-40f6-88bd-80e5f238983a}</author>
+    <author>tc={716b3b85-742b-4e3a-b89f-5b5a3dce4a2c}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{22a33020-94ca-405d-b52d-f5563f0938a4}" ref="E1">
+    <comment authorId="0" xr:uid="{04b0f02b-9ddd-40f6-88bd-80e5f238983a}" ref="E1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -28,7 +28,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{32d35ea2-5a02-472b-9436-72eda681c8bd}" ref="B1">
+    <comment authorId="1" xr:uid="{716b3b85-742b-4e3a-b89f-5b5a3dce4a2c}" ref="B1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="131">
   <si>
     <t>ID</t>
   </si>
@@ -323,9 +323,6 @@
     <t>Módulo de asignación de mano de obra</t>
   </si>
   <si>
-    <t>En Progreso</t>
-  </si>
-  <si>
     <t>Asignación de tareas por trabajador (visualización de los pedidos asignados)</t>
   </si>
   <si>
@@ -353,31 +350,31 @@
     <t>Validacion pruebas Sprint 2</t>
   </si>
   <si>
+    <t>Reunión de avance y validación con el cliente (Sprint 2)</t>
+  </si>
+  <si>
+    <t>Validación de Sprint 2</t>
+  </si>
+  <si>
+    <t>Integración de mapa interactivo</t>
+  </si>
+  <si>
+    <t>Mapa de la dirección del taller en la landing page</t>
+  </si>
+  <si>
+    <t>Integración con API de Google Calendar para fechas límite</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+  </si>
+  <si>
+    <t>H-1</t>
+  </si>
+  <si>
+    <t>Logica integracion con Google Calendar</t>
+  </si>
+  <si>
     <t>Sin Empezar</t>
-  </si>
-  <si>
-    <t>Reunión de avance y validación con el cliente (Sprint 2)</t>
-  </si>
-  <si>
-    <t>Validación de Sprint 2</t>
-  </si>
-  <si>
-    <t>Integración de mapa interactivo</t>
-  </si>
-  <si>
-    <t>Mapa de la dirección del taller en la landing page</t>
-  </si>
-  <si>
-    <t>Integración con API de Google Calendar para fechas límite</t>
-  </si>
-  <si>
-    <t>Sprint 3</t>
-  </si>
-  <si>
-    <t>H-1</t>
-  </si>
-  <si>
-    <t>Logica integracion con Google Calendar</t>
   </si>
   <si>
     <t>Desarrollo integracion backend del Dashboard</t>
@@ -515,7 +512,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="SMOLENKS JOHAN ARAVENA CARVAJAL" id="{fbfe4390-fc9b-46e4-aabe-2d249994f862}" providerId="google-sheets"/>
+  <x18tc:person displayName="SMOLENKS JOHAN ARAVENA CARVAJAL" id="{c6f28ad7-302e-4041-be19-bd82af52f826}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -715,10 +712,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="B1" dT="2026-09-13T21:27:38.00" personId="{fbfe4390-fc9b-46e4-aabe-2d249994f862}" id="{32d35ea2-5a02-472b-9436-72eda681c8bd}" done="1">
+  <x18tc:threadedComment ref="B1" dT="2026-09-13T21:27:38.00" personId="{c6f28ad7-302e-4041-be19-bd82af52f826}" id="{716b3b85-742b-4e3a-b89f-5b5a3dce4a2c}" done="1">
     <x18tc:text xml:space="preserve">eliminar los que no aplican y cambiar redaccion</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="E1" dT="2026-09-13T21:27:43.00" personId="{fbfe4390-fc9b-46e4-aabe-2d249994f862}" id="{22a33020-94ca-405d-b52d-f5563f0938a4}" done="1">
+  <x18tc:threadedComment ref="E1" dT="2026-09-13T21:27:43.00" personId="{c6f28ad7-302e-4041-be19-bd82af52f826}" id="{04b0f02b-9ddd-40f6-88bd-80e5f238983a}" done="1">
     <x18tc:text xml:space="preserve">eliminar los que no aplican y cambiar redaccion</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -1655,7 +1652,7 @@
         <v>12</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>93</v>
+        <v>13</v>
       </c>
       <c r="H33" s="3">
         <f t="shared" si="2"/>
@@ -1668,16 +1665,16 @@
         <v>P-33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>73</v>
       </c>
       <c r="D34" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>95</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>96</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>20</v>
@@ -1696,7 +1693,7 @@
         <v>P-34</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>73</v>
@@ -1705,13 +1702,13 @@
         <v>10</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>93</v>
+        <v>13</v>
       </c>
       <c r="H35" s="3">
         <f t="shared" si="2"/>
@@ -1724,7 +1721,7 @@
         <v>P-35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>73</v>
@@ -1733,13 +1730,13 @@
         <v>10</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>93</v>
+        <v>13</v>
       </c>
       <c r="H36" s="3">
         <f t="shared" si="2"/>
@@ -1752,7 +1749,7 @@
         <v>P-36</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>73</v>
@@ -1761,13 +1758,13 @@
         <v>10</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>103</v>
+        <v>13</v>
       </c>
       <c r="H37" s="3">
         <f t="shared" si="2"/>
@@ -1780,7 +1777,7 @@
         <v>P-37</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>73</v>
@@ -1789,13 +1786,13 @@
         <v>10</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>103</v>
+        <v>13</v>
       </c>
       <c r="H38" s="3">
         <f t="shared" si="2"/>
@@ -1808,7 +1805,7 @@
         <v>P-38</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>73</v>
@@ -1817,7 +1814,7 @@
         <v>10</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>20</v>
@@ -1836,22 +1833,22 @@
         <v>P-39</v>
       </c>
       <c r="B40" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D40" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="E40" s="3" t="s">
         <v>109</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>111</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>20</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="H40" s="3">
         <f t="shared" si="2"/>
@@ -1864,22 +1861,22 @@
         <v>P-40</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D41" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C41" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D41" s="3" t="s">
+      <c r="E41" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="E41" s="3" t="s">
-        <v>114</v>
-      </c>
       <c r="F41" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="H41" s="3">
         <f t="shared" si="2"/>
@@ -1892,22 +1889,22 @@
         <v>P-41</v>
       </c>
       <c r="B42" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E42" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="C42" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>116</v>
-      </c>
       <c r="F42" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="H42" s="3">
         <f t="shared" si="2"/>
@@ -1920,22 +1917,22 @@
         <v>P-42</v>
       </c>
       <c r="B43" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E43" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="C43" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>118</v>
-      </c>
       <c r="F43" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="H43" s="3">
         <f t="shared" si="2"/>
@@ -1948,22 +1945,22 @@
         <v>P-43</v>
       </c>
       <c r="B44" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E44" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C44" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>120</v>
-      </c>
       <c r="F44" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="H44" s="3">
         <f t="shared" si="2"/>
@@ -1976,22 +1973,22 @@
         <v>P-44</v>
       </c>
       <c r="B45" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E45" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="C45" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E45" s="3" t="s">
-        <v>122</v>
-      </c>
       <c r="F45" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="H45" s="3">
         <f t="shared" si="2"/>
@@ -2004,22 +2001,22 @@
         <v>P-45</v>
       </c>
       <c r="B46" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C46" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="D46" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E46" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D46" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E46" s="3" t="s">
-        <v>125</v>
-      </c>
       <c r="F46" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="H46" s="3">
         <f t="shared" si="2"/>
@@ -2032,22 +2029,22 @@
         <v>P-46</v>
       </c>
       <c r="B47" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E47" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C47" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="D47" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E47" s="3" t="s">
-        <v>127</v>
-      </c>
       <c r="F47" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="H47" s="3">
         <f t="shared" si="2"/>
@@ -2060,22 +2057,22 @@
         <v>P-47</v>
       </c>
       <c r="B48" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E48" s="3" t="s">
         <v>128</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>129</v>
       </c>
       <c r="F48" s="3" t="s">
         <v>20</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="H48" s="3">
         <f t="shared" si="2"/>
@@ -2088,22 +2085,22 @@
         <v>P-48</v>
       </c>
       <c r="B49" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E49" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="C49" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>131</v>
-      </c>
       <c r="F49" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="H49" s="3">
         <f t="shared" si="2"/>

</xml_diff>